<commit_message>
Rebuild every output against the remetriced corpus
Notebooks 1, 2 and 3 run end to end with no errors and no warnings.
TABLE_PLCAResults.csv is byte-identical to the previous run, which is the
check that the remetric changed no data; the tables that move are the ones
carrying weight_outliers or derived from it, plus every figure rebuilt on
the corrected axis scaling.

Twelve new per-characteristic supplement figures.

Co-Authored-By: Claude Opus 5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/outputs/tables/TABLE_EmpiricalECCMetrics.xlsx
+++ b/outputs/tables/TABLE_EmpiricalECCMetrics.xlsx
@@ -1751,10 +1751,10 @@
         <v>0.09293681618496408</v>
       </c>
       <c r="V18" t="n">
-        <v>0</v>
+        <v>0.3622193416706191</v>
       </c>
       <c r="W18" t="n">
-        <v>0</v>
+        <v>0.3333333333333333</v>
       </c>
     </row>
     <row r="19">
@@ -4736,7 +4736,7 @@
         <v>0.009230255466642488</v>
       </c>
       <c r="V59" t="n">
-        <v>0</v>
+        <v>0.2482240629063026</v>
       </c>
       <c r="W59" t="n">
         <v>0</v>
@@ -11229,7 +11229,7 @@
         <v>0.2444793042576891</v>
       </c>
       <c r="V148" t="n">
-        <v>0</v>
+        <v>0.01969552426254956</v>
       </c>
       <c r="W148" t="n">
         <v>0.1428571428571428</v>

</xml_diff>

<commit_message>
Rerun at Silverman divisor 1.35, part 2 of 3: remaining tables (decision 260)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/outputs/tables/TABLE_EmpiricalECCMetrics.xlsx
+++ b/outputs/tables/TABLE_EmpiricalECCMetrics.xlsx
@@ -593,7 +593,7 @@
         <v>1.001005137361129</v>
       </c>
       <c r="R2" t="n">
-        <v>1.040928943346033</v>
+        <v>1.041371815820066</v>
       </c>
       <c r="S2" t="n">
         <v>1.028084151618127</v>
@@ -748,10 +748,10 @@
         <v>1.016773947613548</v>
       </c>
       <c r="Q4" t="n">
-        <v>1.117779760793197</v>
+        <v>1.118913806324753</v>
       </c>
       <c r="R4" t="n">
-        <v>1.074827170779614</v>
+        <v>1.075796374591005</v>
       </c>
       <c r="S4" t="n">
         <v>1.008822288055942</v>
@@ -827,10 +827,10 @@
         <v>1.005306417188222</v>
       </c>
       <c r="Q5" t="n">
-        <v>1.135991607168941</v>
+        <v>1.136143049127039</v>
       </c>
       <c r="R5" t="n">
-        <v>1.106463291044453</v>
+        <v>1.106519789666069</v>
       </c>
       <c r="S5" t="n">
         <v>1.005654889400433</v>
@@ -909,7 +909,7 @@
         <v>1.017960331410465</v>
       </c>
       <c r="R6" t="n">
-        <v>1.034609716389288</v>
+        <v>1.035644061647895</v>
       </c>
       <c r="S6" t="n">
         <v>1.017329270759607</v>
@@ -988,7 +988,7 @@
         <v>1.014211249708263</v>
       </c>
       <c r="R7" t="n">
-        <v>1.159210556004727</v>
+        <v>1.161841353784153</v>
       </c>
       <c r="S7" t="n">
         <v>1.070504973760363</v>
@@ -1067,7 +1067,7 @@
         <v>1</v>
       </c>
       <c r="R8" t="n">
-        <v>1.003307479763752</v>
+        <v>1.004320645346087</v>
       </c>
       <c r="S8" t="n">
         <v>1</v>
@@ -1221,7 +1221,7 @@
         <v>1.060612924990478</v>
       </c>
       <c r="R10" t="n">
-        <v>1.094247496742057</v>
+        <v>1.097297761196359</v>
       </c>
       <c r="S10" t="n">
         <v>1.020400589490248</v>
@@ -1297,10 +1297,10 @@
         <v>1.013475204322204</v>
       </c>
       <c r="Q11" t="n">
-        <v>1.028614414198721</v>
+        <v>1.028935613387999</v>
       </c>
       <c r="R11" t="n">
-        <v>1.025951272610127</v>
+        <v>1.026258495497775</v>
       </c>
       <c r="S11" t="n">
         <v>1.009154565156715</v>
@@ -1376,10 +1376,10 @@
         <v>1.080549448342853</v>
       </c>
       <c r="Q12" t="n">
-        <v>1.201758612243786</v>
+        <v>1.204092102131916</v>
       </c>
       <c r="R12" t="n">
-        <v>1.137314367612276</v>
+        <v>1.13972238004452</v>
       </c>
       <c r="S12" t="n">
         <v>1.037033785089428</v>
@@ -1455,10 +1455,10 @@
         <v>1.029396277306996</v>
       </c>
       <c r="Q13" t="n">
-        <v>1.114368293052237</v>
+        <v>1.115693451104787</v>
       </c>
       <c r="R13" t="n">
-        <v>1.049153364533274</v>
+        <v>1.049770517554048</v>
       </c>
       <c r="S13" t="n">
         <v>1.022207261993878</v>
@@ -1537,7 +1537,7 @@
         <v>1.04743179209658</v>
       </c>
       <c r="R14" t="n">
-        <v>1.095848139130641</v>
+        <v>1.096486527360492</v>
       </c>
       <c r="S14" t="n">
         <v>1.060576411318667</v>
@@ -1613,10 +1613,10 @@
         <v>1.048655536058486</v>
       </c>
       <c r="Q15" t="n">
-        <v>1.059818382507851</v>
+        <v>1.06064613716609</v>
       </c>
       <c r="R15" t="n">
-        <v>1.098512757175423</v>
+        <v>1.0998850446617</v>
       </c>
       <c r="S15" t="n">
         <v>1.053545989607294</v>
@@ -1767,10 +1767,10 @@
         <v>1.001928862956075</v>
       </c>
       <c r="Q17" t="n">
-        <v>1.067589308846356</v>
+        <v>1.069352440673402</v>
       </c>
       <c r="R17" t="n">
-        <v>1.090605257640002</v>
+        <v>1.091878950776468</v>
       </c>
       <c r="S17" t="n">
         <v>1.012983759217844</v>
@@ -2000,10 +2000,10 @@
         <v>1.054261395994039</v>
       </c>
       <c r="Q20" t="n">
-        <v>1.183176781354193</v>
+        <v>1.185236522835171</v>
       </c>
       <c r="R20" t="n">
-        <v>1.093883842034411</v>
+        <v>1.09488092595851</v>
       </c>
       <c r="S20" t="n">
         <v>1.028183096469301</v>
@@ -2082,7 +2082,7 @@
         <v>1.013474520786705</v>
       </c>
       <c r="R21" t="n">
-        <v>1.102597468904421</v>
+        <v>1.10342149137605</v>
       </c>
       <c r="S21" t="n">
         <v>1.040669813376224</v>
@@ -2237,10 +2237,10 @@
         <v>1.003368971976756</v>
       </c>
       <c r="Q23" t="n">
-        <v>1.058232584769141</v>
+        <v>1.058955408914242</v>
       </c>
       <c r="R23" t="n">
-        <v>1.064295313634011</v>
+        <v>1.064910610970679</v>
       </c>
       <c r="S23" t="n">
         <v>1.020510203801384</v>
@@ -2395,10 +2395,10 @@
         <v>1.001474574675983</v>
       </c>
       <c r="Q25" t="n">
-        <v>1.024118723169152</v>
+        <v>1.024365295147244</v>
       </c>
       <c r="R25" t="n">
-        <v>1.00044850973277</v>
+        <v>1.000594388582842</v>
       </c>
       <c r="S25" t="n">
         <v>1</v>
@@ -2474,10 +2474,10 @@
         <v>1.022644424446105</v>
       </c>
       <c r="Q26" t="n">
-        <v>1.111093477678355</v>
+        <v>1.111770225505706</v>
       </c>
       <c r="R26" t="n">
-        <v>1.146520993992054</v>
+        <v>1.147915825999789</v>
       </c>
       <c r="S26" t="n">
         <v>1.020311499581628</v>
@@ -2553,10 +2553,10 @@
         <v>1</v>
       </c>
       <c r="Q27" t="n">
-        <v>1.066517157184333</v>
+        <v>1.070447850305662</v>
       </c>
       <c r="R27" t="n">
-        <v>1</v>
+        <v>1.000064240997709</v>
       </c>
       <c r="S27" t="n">
         <v>1</v>
@@ -2790,10 +2790,10 @@
         <v>1.005232062798919</v>
       </c>
       <c r="Q30" t="n">
-        <v>1.013401556433007</v>
+        <v>1.013570778072815</v>
       </c>
       <c r="R30" t="n">
-        <v>1.016649198754034</v>
+        <v>1.017572587536853</v>
       </c>
       <c r="S30" t="n">
         <v>1.004047425114218</v>
@@ -2951,7 +2951,7 @@
         <v>1.00565550153298</v>
       </c>
       <c r="R32" t="n">
-        <v>1.089840870387961</v>
+        <v>1.094016768518122</v>
       </c>
       <c r="S32" t="n">
         <v>1.02100698543268</v>
@@ -3027,10 +3027,10 @@
         <v>1.008108801711226</v>
       </c>
       <c r="Q33" t="n">
-        <v>1.025978438358032</v>
+        <v>1.026398670056827</v>
       </c>
       <c r="R33" t="n">
-        <v>1.123139887123249</v>
+        <v>1.127000157449258</v>
       </c>
       <c r="S33" t="n">
         <v>1.035324952445202</v>
@@ -3106,7 +3106,7 @@
         <v>1</v>
       </c>
       <c r="Q34" t="n">
-        <v>1.000025206500891</v>
+        <v>1.00002686342504</v>
       </c>
       <c r="R34" t="n">
         <v>1.011916826192858</v>
@@ -3185,7 +3185,7 @@
         <v>1.000279273016993</v>
       </c>
       <c r="Q35" t="n">
-        <v>1.006796332644302</v>
+        <v>1.007290045400148</v>
       </c>
       <c r="R35" t="n">
         <v>1.012689686580874</v>
@@ -3264,10 +3264,10 @@
         <v>1.007528792011665</v>
       </c>
       <c r="Q36" t="n">
-        <v>1.02119732637524</v>
+        <v>1.021835127900505</v>
       </c>
       <c r="R36" t="n">
-        <v>1.013873069787575</v>
+        <v>1.014142832617421</v>
       </c>
       <c r="S36" t="n">
         <v>1.007902376243321</v>
@@ -3346,7 +3346,7 @@
         <v>1.164500580507336</v>
       </c>
       <c r="R37" t="n">
-        <v>1.08355843659071</v>
+        <v>1.087129837971888</v>
       </c>
       <c r="S37" t="n">
         <v>1</v>
@@ -3422,10 +3422,10 @@
         <v>1.006818309509078</v>
       </c>
       <c r="Q38" t="n">
-        <v>1.0150309908208</v>
+        <v>1.015500751504483</v>
       </c>
       <c r="R38" t="n">
-        <v>1.026112799374688</v>
+        <v>1.026685062060117</v>
       </c>
       <c r="S38" t="n">
         <v>1.006566987101052</v>
@@ -3580,10 +3580,10 @@
         <v>1.017003241003839</v>
       </c>
       <c r="Q40" t="n">
-        <v>1.034011606644861</v>
+        <v>1.036009599883016</v>
       </c>
       <c r="R40" t="n">
-        <v>1.09145096882896</v>
+        <v>1.095038354494908</v>
       </c>
       <c r="S40" t="n">
         <v>1.016613509646723</v>
@@ -3813,10 +3813,10 @@
         <v>1.009466591963998</v>
       </c>
       <c r="Q43" t="n">
-        <v>1.084583491593362</v>
+        <v>1.084964957231459</v>
       </c>
       <c r="R43" t="n">
-        <v>1.047501299852954</v>
+        <v>1.048384377869743</v>
       </c>
       <c r="S43" t="n">
         <v>1.009314532090233</v>
@@ -3974,7 +3974,7 @@
         <v>1.112796744487812</v>
       </c>
       <c r="R45" t="n">
-        <v>1.002564935690344</v>
+        <v>1.003500405524472</v>
       </c>
       <c r="S45" t="n">
         <v>1</v>
@@ -4211,7 +4211,7 @@
         <v>1.193671307438383</v>
       </c>
       <c r="R48" t="n">
-        <v>1.140283965988981</v>
+        <v>1.143732994453072</v>
       </c>
       <c r="S48" t="n">
         <v>1.07071058825641</v>
@@ -4290,7 +4290,7 @@
         <v>1.047403668878102</v>
       </c>
       <c r="R49" t="n">
-        <v>1.056382196913695</v>
+        <v>1.056585979120672</v>
       </c>
       <c r="S49" t="n">
         <v>1.047719077478554</v>
@@ -4366,10 +4366,10 @@
         <v>1.044027435087589</v>
       </c>
       <c r="Q50" t="n">
-        <v>1.060968474854467</v>
+        <v>1.061375837601876</v>
       </c>
       <c r="R50" t="n">
-        <v>1.064229761868608</v>
+        <v>1.065551599416964</v>
       </c>
       <c r="S50" t="n">
         <v>1.020328607656752</v>
@@ -4445,10 +4445,10 @@
         <v>1.03071495916729</v>
       </c>
       <c r="Q51" t="n">
-        <v>1.108714477349759</v>
+        <v>1.109515923361111</v>
       </c>
       <c r="R51" t="n">
-        <v>1.144649805670209</v>
+        <v>1.146002786956885</v>
       </c>
       <c r="S51" t="n">
         <v>1.023438953331128</v>
@@ -4524,10 +4524,10 @@
         <v>1.009637718721611</v>
       </c>
       <c r="Q52" t="n">
-        <v>1.023846426141057</v>
+        <v>1.023987241206366</v>
       </c>
       <c r="R52" t="n">
-        <v>1.055061851730484</v>
+        <v>1.055754558196295</v>
       </c>
       <c r="S52" t="n">
         <v>1.009498219147334</v>
@@ -4682,10 +4682,10 @@
         <v>1.000928172842933</v>
       </c>
       <c r="Q54" t="n">
-        <v>1.100211466831979</v>
+        <v>1.101927690068251</v>
       </c>
       <c r="R54" t="n">
-        <v>1.097390961791228</v>
+        <v>1.100179195723765</v>
       </c>
       <c r="S54" t="n">
         <v>1.005950304274737</v>
@@ -4919,10 +4919,10 @@
         <v>1.010334977323024</v>
       </c>
       <c r="Q57" t="n">
-        <v>1.032153325114691</v>
+        <v>1.03240040044616</v>
       </c>
       <c r="R57" t="n">
-        <v>1.119521690979794</v>
+        <v>1.121337249992476</v>
       </c>
       <c r="S57" t="n">
         <v>1.025420395412684</v>
@@ -5076,7 +5076,7 @@
         <v>1.083716170495417</v>
       </c>
       <c r="R59" t="n">
-        <v>1.241365995508224</v>
+        <v>1.242313264637713</v>
       </c>
       <c r="S59" t="n">
         <v>1.053539405537984</v>
@@ -5231,10 +5231,10 @@
         <v>1.003257632254175</v>
       </c>
       <c r="Q61" t="n">
-        <v>1.015930975536776</v>
+        <v>1.016565413489855</v>
       </c>
       <c r="R61" t="n">
-        <v>1.041323597038271</v>
+        <v>1.042621615051056</v>
       </c>
       <c r="S61" t="n">
         <v>1.007126677254597</v>
@@ -5313,7 +5313,7 @@
         <v>1.038206103802567</v>
       </c>
       <c r="R62" t="n">
-        <v>1.09524882328101</v>
+        <v>1.095233475569031</v>
       </c>
       <c r="S62" t="n">
         <v>1.063776019084027</v>
@@ -5392,7 +5392,7 @@
         <v>1.096863075106416</v>
       </c>
       <c r="R63" t="n">
-        <v>1.215258947895359</v>
+        <v>1.219112277842685</v>
       </c>
       <c r="S63" t="n">
         <v>1.039811505058307</v>
@@ -5550,7 +5550,7 @@
         <v>1.008501710306724</v>
       </c>
       <c r="R65" t="n">
-        <v>1.070308258708538</v>
+        <v>1.071213945610821</v>
       </c>
       <c r="S65" t="n">
         <v>1.031453791401421</v>
@@ -5626,10 +5626,10 @@
         <v>1.010849983984087</v>
       </c>
       <c r="Q66" t="n">
-        <v>1.021642759681015</v>
+        <v>1.021912895320703</v>
       </c>
       <c r="R66" t="n">
-        <v>1.044157757569472</v>
+        <v>1.044708832486122</v>
       </c>
       <c r="S66" t="n">
         <v>1.015013990405764</v>
@@ -5942,10 +5942,10 @@
         <v>1.052465911252749</v>
       </c>
       <c r="Q70" t="n">
-        <v>1.08102935277936</v>
+        <v>1.08156199152313</v>
       </c>
       <c r="R70" t="n">
-        <v>1.037034672543807</v>
+        <v>1.037384215505138</v>
       </c>
       <c r="S70" t="n">
         <v>1.023207025568986</v>
@@ -6021,10 +6021,10 @@
         <v>1.01250487802955</v>
       </c>
       <c r="Q71" t="n">
-        <v>1.026156448743483</v>
+        <v>1.026353246044601</v>
       </c>
       <c r="R71" t="n">
-        <v>1.029419651223312</v>
+        <v>1.029702678114278</v>
       </c>
       <c r="S71" t="n">
         <v>1.012630819694899</v>
@@ -6337,10 +6337,10 @@
         <v>1.01915392111379</v>
       </c>
       <c r="Q75" t="n">
-        <v>1.183325607898676</v>
+        <v>1.184003819840244</v>
       </c>
       <c r="R75" t="n">
-        <v>1.299183612446371</v>
+        <v>1.30103486506603</v>
       </c>
       <c r="S75" t="n">
         <v>1.035419072932095</v>
@@ -6416,10 +6416,10 @@
         <v>1.033475854842358</v>
       </c>
       <c r="Q76" t="n">
-        <v>1.083085134862351</v>
+        <v>1.084752210383922</v>
       </c>
       <c r="R76" t="n">
-        <v>1.01472471618983</v>
+        <v>1.015188617681806</v>
       </c>
       <c r="S76" t="n">
         <v>1.00935474362358</v>
@@ -6495,10 +6495,10 @@
         <v>1.010086023593949</v>
       </c>
       <c r="Q77" t="n">
-        <v>1.013758140317791</v>
+        <v>1.013841681361958</v>
       </c>
       <c r="R77" t="n">
-        <v>1.008408193453572</v>
+        <v>1.008466247582792</v>
       </c>
       <c r="S77" t="n">
         <v>1.006702423634908</v>
@@ -6577,7 +6577,7 @@
         <v>1.000105927208099</v>
       </c>
       <c r="R78" t="n">
-        <v>1.139678607190467</v>
+        <v>1.140490649595412</v>
       </c>
       <c r="S78" t="n">
         <v>1.006423424039746</v>
@@ -6814,7 +6814,7 @@
         <v>1.085063658874821</v>
       </c>
       <c r="R81" t="n">
-        <v>1.098696964806258</v>
+        <v>1.099623643501167</v>
       </c>
       <c r="S81" t="n">
         <v>1.025866133362981</v>
@@ -6893,7 +6893,7 @@
         <v>1.008399520679616</v>
       </c>
       <c r="R82" t="n">
-        <v>1.05127383074672</v>
+        <v>1.052841477046448</v>
       </c>
       <c r="S82" t="n">
         <v>1</v>
@@ -6969,10 +6969,10 @@
         <v>1.10023898526898</v>
       </c>
       <c r="Q83" t="n">
-        <v>1.227149875949632</v>
+        <v>1.227728040334726</v>
       </c>
       <c r="R83" t="n">
-        <v>1.190435449306315</v>
+        <v>1.19126269922003</v>
       </c>
       <c r="S83" t="n">
         <v>1.096834633890862</v>
@@ -7051,7 +7051,7 @@
         <v>1.001577046792815</v>
       </c>
       <c r="R84" t="n">
-        <v>1.162644459024371</v>
+        <v>1.164813175855732</v>
       </c>
       <c r="S84" t="n">
         <v>1.016696448388154</v>
@@ -7130,7 +7130,7 @@
         <v>1.018685932803797</v>
       </c>
       <c r="R85" t="n">
-        <v>1.063993467385989</v>
+        <v>1.065899030805943</v>
       </c>
       <c r="S85" t="n">
         <v>1.023267504114854</v>
@@ -7443,10 +7443,10 @@
         <v>1.036823526797908</v>
       </c>
       <c r="Q89" t="n">
-        <v>1.130853435263917</v>
+        <v>1.13381697196313</v>
       </c>
       <c r="R89" t="n">
-        <v>1.056052410512879</v>
+        <v>1.059491866107141</v>
       </c>
       <c r="S89" t="n">
         <v>1.022144060724332</v>
@@ -7522,10 +7522,10 @@
         <v>1.016675447209708</v>
       </c>
       <c r="Q90" t="n">
-        <v>1.066650411213881</v>
+        <v>1.067414600117276</v>
       </c>
       <c r="R90" t="n">
-        <v>1.098162439654083</v>
+        <v>1.0988971811051</v>
       </c>
       <c r="S90" t="n">
         <v>1.022418497241333</v>
@@ -7683,7 +7683,7 @@
         <v>1.015491839119834</v>
       </c>
       <c r="R92" t="n">
-        <v>1.127756234512661</v>
+        <v>1.129756875595182</v>
       </c>
       <c r="S92" t="n">
         <v>1.000255009972166</v>
@@ -7762,7 +7762,7 @@
         <v>1.009574733636376</v>
       </c>
       <c r="R93" t="n">
-        <v>1.088386244467616</v>
+        <v>1.091325654718282</v>
       </c>
       <c r="S93" t="n">
         <v>1.033688772809744</v>
@@ -7838,10 +7838,10 @@
         <v>1.017525371528395</v>
       </c>
       <c r="Q94" t="n">
-        <v>1.132920330374832</v>
+        <v>1.134441569559192</v>
       </c>
       <c r="R94" t="n">
-        <v>1.165732751759302</v>
+        <v>1.169218555655489</v>
       </c>
       <c r="S94" t="n">
         <v>1.039029327919982</v>
@@ -8075,10 +8075,10 @@
         <v>1.014104428106125</v>
       </c>
       <c r="Q97" t="n">
-        <v>1.034277594365932</v>
+        <v>1.034829752274044</v>
       </c>
       <c r="R97" t="n">
-        <v>1.049673764268197</v>
+        <v>1.050741589488603</v>
       </c>
       <c r="S97" t="n">
         <v>1.0090969367735</v>
@@ -8233,10 +8233,10 @@
         <v>1.016251206873568</v>
       </c>
       <c r="Q99" t="n">
-        <v>1.040146902911874</v>
+        <v>1.040664163486428</v>
       </c>
       <c r="R99" t="n">
-        <v>1.121475256785471</v>
+        <v>1.125190571316243</v>
       </c>
       <c r="S99" t="n">
         <v>1.036482101907221</v>
@@ -8315,7 +8315,7 @@
         <v>1</v>
       </c>
       <c r="R100" t="n">
-        <v>1.020167778469986</v>
+        <v>1.021258290171881</v>
       </c>
       <c r="S100" t="n">
         <v>1.000858196647481</v>
@@ -8391,10 +8391,10 @@
         <v>1.017535480649453</v>
       </c>
       <c r="Q101" t="n">
-        <v>1.095040746556481</v>
+        <v>1.0960638649596</v>
       </c>
       <c r="R101" t="n">
-        <v>1.082533642224376</v>
+        <v>1.083347527794401</v>
       </c>
       <c r="S101" t="n">
         <v>1.013484922788592</v>
@@ -8470,10 +8470,10 @@
         <v>1.009097458874169</v>
       </c>
       <c r="Q102" t="n">
-        <v>1.040510312661889</v>
+        <v>1.041459514564951</v>
       </c>
       <c r="R102" t="n">
-        <v>1.051552741916877</v>
+        <v>1.053115674218995</v>
       </c>
       <c r="S102" t="n">
         <v>1.015071317116978</v>
@@ -8549,10 +8549,10 @@
         <v>1.010879044614635</v>
       </c>
       <c r="Q103" t="n">
-        <v>1.044967177118566</v>
+        <v>1.045614230738552</v>
       </c>
       <c r="R103" t="n">
-        <v>1.047314072748331</v>
+        <v>1.047660121784866</v>
       </c>
       <c r="S103" t="n">
         <v>1.020541475120251</v>
@@ -8628,10 +8628,10 @@
         <v>1.000745040550296</v>
       </c>
       <c r="Q104" t="n">
-        <v>1.001455952920771</v>
+        <v>1.001512663626723</v>
       </c>
       <c r="R104" t="n">
-        <v>1.001772487326929</v>
+        <v>1.00182708648815</v>
       </c>
       <c r="S104" t="n">
         <v>1.000830925627947</v>
@@ -8707,10 +8707,10 @@
         <v>1.001446298869981</v>
       </c>
       <c r="Q105" t="n">
-        <v>1.002652126390932</v>
+        <v>1.002668142936662</v>
       </c>
       <c r="R105" t="n">
-        <v>1.00250265881513</v>
+        <v>1.002522392830705</v>
       </c>
       <c r="S105" t="n">
         <v>1.001944668362955</v>
@@ -8865,10 +8865,10 @@
         <v>1.007528808882736</v>
       </c>
       <c r="Q107" t="n">
-        <v>1.011366143999975</v>
+        <v>1.011830704961316</v>
       </c>
       <c r="R107" t="n">
-        <v>1.017536230417437</v>
+        <v>1.017791839749926</v>
       </c>
       <c r="S107" t="n">
         <v>1.00994527209299</v>
@@ -9023,10 +9023,10 @@
         <v>1.002013807548805</v>
       </c>
       <c r="Q109" t="n">
-        <v>1.003714004434963</v>
+        <v>1.003796442919276</v>
       </c>
       <c r="R109" t="n">
-        <v>1.007795364176455</v>
+        <v>1.008279082668069</v>
       </c>
       <c r="S109" t="n">
         <v>1.003893016525779</v>
@@ -9102,10 +9102,10 @@
         <v>1.014687776985438</v>
       </c>
       <c r="Q110" t="n">
-        <v>1.142899371814483</v>
+        <v>1.144445338953628</v>
       </c>
       <c r="R110" t="n">
-        <v>1.112001908521034</v>
+        <v>1.112791113416083</v>
       </c>
       <c r="S110" t="n">
         <v>1.025271466101481</v>
@@ -9181,10 +9181,10 @@
         <v>1.044217537281513</v>
       </c>
       <c r="Q111" t="n">
-        <v>1.233892375040221</v>
+        <v>1.2374806507151</v>
       </c>
       <c r="R111" t="n">
-        <v>1.137409975552358</v>
+        <v>1.13955957646049</v>
       </c>
       <c r="S111" t="n">
         <v>1.037810624895072</v>
@@ -9263,7 +9263,7 @@
         <v>1</v>
       </c>
       <c r="R112" t="n">
-        <v>1.020594937432143</v>
+        <v>1.02283463239648</v>
       </c>
       <c r="S112" t="n">
         <v>1</v>
@@ -9342,7 +9342,7 @@
         <v>1.102693387741539</v>
       </c>
       <c r="R113" t="n">
-        <v>1.001984070467864</v>
+        <v>1.002290808304046</v>
       </c>
       <c r="S113" t="n">
         <v>1</v>
@@ -9418,10 +9418,10 @@
         <v>1.006012606692849</v>
       </c>
       <c r="Q114" t="n">
-        <v>1.329854565967702</v>
+        <v>1.332158884173532</v>
       </c>
       <c r="R114" t="n">
-        <v>1.052413834280961</v>
+        <v>1.053861813538904</v>
       </c>
       <c r="S114" t="n">
         <v>1.00123504297487</v>
@@ -9500,7 +9500,7 @@
         <v>1.002098553553409</v>
       </c>
       <c r="R115" t="n">
-        <v>1.029799443504566</v>
+        <v>1.03112065460028</v>
       </c>
       <c r="S115" t="n">
         <v>1.004505860103953</v>
@@ -9576,10 +9576,10 @@
         <v>1</v>
       </c>
       <c r="Q116" t="n">
-        <v>1.028423280103563</v>
+        <v>1.031202497954827</v>
       </c>
       <c r="R116" t="n">
-        <v>1.000574668343487</v>
+        <v>1.000640374866406</v>
       </c>
       <c r="S116" t="n">
         <v>1</v>
@@ -9813,7 +9813,7 @@
         <v>1</v>
       </c>
       <c r="Q119" t="n">
-        <v>1.00101675698499</v>
+        <v>1.001120070844107</v>
       </c>
       <c r="R119" t="n">
         <v>1.000735000895359</v>
@@ -9892,10 +9892,10 @@
         <v>1.013094761109131</v>
       </c>
       <c r="Q120" t="n">
-        <v>1.132042831740214</v>
+        <v>1.135627244828141</v>
       </c>
       <c r="R120" t="n">
-        <v>1.142472689829257</v>
+        <v>1.143816588786133</v>
       </c>
       <c r="S120" t="n">
         <v>1.062296920709371</v>
@@ -9974,7 +9974,7 @@
         <v>1.014103998890121</v>
       </c>
       <c r="R121" t="n">
-        <v>1.044022486629834</v>
+        <v>1.044722607564978</v>
       </c>
       <c r="S121" t="n">
         <v>1.022020897969908</v>
@@ -10129,10 +10129,10 @@
         <v>1.013149961933713</v>
       </c>
       <c r="Q123" t="n">
-        <v>1.020380669778818</v>
+        <v>1.020622232544045</v>
       </c>
       <c r="R123" t="n">
-        <v>1.047682093341697</v>
+        <v>1.048224754289153</v>
       </c>
       <c r="S123" t="n">
         <v>1.021223614675844</v>
@@ -10211,7 +10211,7 @@
         <v>1.05572362784677</v>
       </c>
       <c r="R124" t="n">
-        <v>1.056555648933941</v>
+        <v>1.057523612713476</v>
       </c>
       <c r="S124" t="n">
         <v>1.045290362191896</v>
@@ -10445,10 +10445,10 @@
         <v>1.013106436406949</v>
       </c>
       <c r="Q127" t="n">
-        <v>1.026421068886595</v>
+        <v>1.026916691563903</v>
       </c>
       <c r="R127" t="n">
-        <v>1.025586231826069</v>
+        <v>1.025750472503384</v>
       </c>
       <c r="S127" t="n">
         <v>1.020658356003813</v>
@@ -10761,10 +10761,10 @@
         <v>1.015075583618936</v>
       </c>
       <c r="Q131" t="n">
-        <v>1.017079013921605</v>
+        <v>1.017163306640877</v>
       </c>
       <c r="R131" t="n">
-        <v>1.069478841464237</v>
+        <v>1.070797261622067</v>
       </c>
       <c r="S131" t="n">
         <v>1.010052084659834</v>
@@ -10840,10 +10840,10 @@
         <v>1.020294196131324</v>
       </c>
       <c r="Q132" t="n">
-        <v>1.126608841608396</v>
+        <v>1.128598743867653</v>
       </c>
       <c r="R132" t="n">
-        <v>1.188453484583632</v>
+        <v>1.190225530849396</v>
       </c>
       <c r="S132" t="n">
         <v>1.028004806138072</v>
@@ -10998,10 +10998,10 @@
         <v>1.046665800453953</v>
       </c>
       <c r="Q134" t="n">
-        <v>1.141421819711912</v>
+        <v>1.14243025552887</v>
       </c>
       <c r="R134" t="n">
-        <v>1.160367896557249</v>
+        <v>1.162515577537538</v>
       </c>
       <c r="S134" t="n">
         <v>1.021736585612737</v>
@@ -11314,10 +11314,10 @@
         <v>1.028656088161708</v>
       </c>
       <c r="Q138" t="n">
-        <v>1.08662541417153</v>
+        <v>1.086909725542303</v>
       </c>
       <c r="R138" t="n">
-        <v>1.091662236116571</v>
+        <v>1.092163920389355</v>
       </c>
       <c r="S138" t="n">
         <v>1.010492619786958</v>
@@ -11393,10 +11393,10 @@
         <v>1.038624047913878</v>
       </c>
       <c r="Q139" t="n">
-        <v>1.124498478724844</v>
+        <v>1.126226182813179</v>
       </c>
       <c r="R139" t="n">
-        <v>1.078373366377271</v>
+        <v>1.07924387306207</v>
       </c>
       <c r="S139" t="n">
         <v>1.033932292630582</v>
@@ -11472,10 +11472,10 @@
         <v>1.020158683026965</v>
       </c>
       <c r="Q140" t="n">
-        <v>1.203888712261839</v>
+        <v>1.204627240844355</v>
       </c>
       <c r="R140" t="n">
-        <v>1.14277074835694</v>
+        <v>1.144111519999631</v>
       </c>
       <c r="S140" t="n">
         <v>1.037569978740648</v>
@@ -11626,10 +11626,10 @@
         <v>1.012582012179135</v>
       </c>
       <c r="Q142" t="n">
-        <v>1.177493547102611</v>
+        <v>1.180410714042639</v>
       </c>
       <c r="R142" t="n">
-        <v>1.097249940681272</v>
+        <v>1.098593285139021</v>
       </c>
       <c r="S142" t="n">
         <v>1.012312089381855</v>
@@ -11705,10 +11705,10 @@
         <v>1.002986794977022</v>
       </c>
       <c r="Q143" t="n">
-        <v>1.049754673128539</v>
+        <v>1.05075406396519</v>
       </c>
       <c r="R143" t="n">
-        <v>1.12562021534747</v>
+        <v>1.126286570838365</v>
       </c>
       <c r="S143" t="n">
         <v>1.037900570163677</v>
@@ -11787,7 +11787,7 @@
         <v>1.012769096579075</v>
       </c>
       <c r="R144" t="n">
-        <v>1.068863888971745</v>
+        <v>1.069762181548098</v>
       </c>
       <c r="S144" t="n">
         <v>1.000278931611801</v>
@@ -11863,10 +11863,10 @@
         <v>1.017775406722974</v>
       </c>
       <c r="Q145" t="n">
-        <v>1.173608048918247</v>
+        <v>1.175835024156027</v>
       </c>
       <c r="R145" t="n">
-        <v>1.076126932884518</v>
+        <v>1.077475759745978</v>
       </c>
       <c r="S145" t="n">
         <v>1.000144120413532</v>

</xml_diff>